<commit_message>
Session 101 Task 1: Missouri SMRP priced, $34,646,479.34; DSS26015-02 closed, outcome unknown
DSS's SMRP page now reads 'A full list of awardees and allocation is
below' over an 'RHTP | Awarded Amount' table: awarded amounts, not
maximums or requests. The 20 hospital rows are rewritten from it (sum
asserted to the cent; no total printed). Programme page, SMRP page and
bid table archived 2026-10-15 and re-based; prior copies kept.
IFB DSS26015-02 is off the bid table with no outcome published: recorded
CLOSED_OUTCOME_UNKNOWN, and the bid check is now an award watch (fires on
its reappearance or award wording). Kids Win Missouri and the MU CNM
contract (the 10-14 name trip) are read, non-hospital, and not extracted.
Cross-file partition pins are updated later this session.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LynoGSXHyfySsNBiQ3QjWs
</commit_message>
<xml_diff>
--- a/MO_year1_awardees.xlsx
+++ b/MO_year1_awardees.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t xml:space="preserve">MISSOURI HAS PUBLISHED A 27-ORGANISATION ROSTER AND TWO AWARDS. THEY ARE NOT THE SAME THING.</t>
   </si>
@@ -41,25 +41,28 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">Missouri's award actions are the TWO on sheet 'Awards': the Missouri Doula Association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">($732,660.43, exact) and the Missouri EMS Association (around $6.5M, running through 2027-07-31).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both are pass-through administrators; neither reaches a hospital. MISSOURI'S NAMED-HOSPITAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOLLARS ARE $0, and that is a statement about what DSS has published, not about Missouri.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The hospital money is coming through PROCUREMENT: the ToRCH Care Smart Growth IFB anticipates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nearly $40M with individual awards up to $5M, open to hospitals, and DSS's own timeline says</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Aug - Sept 2026 Announce select procurement awardees'. None had been announced when this was built.</t>
+    <t xml:space="preserve">Missouri's award actions are the 22 on sheet 'Awards': the Missouri Doula Association</t>
+  </si>
+  <si>
+    <t xml:space="preserve">($732,660.43, exact), the Missouri EMS Association (around $6.5M, running through 2027-07-31),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">both pass-through administrators that do not reach a hospital, and the TWENTY Strategic Minor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renovations Program hospital awards, priced by DSS on its own page at $34,646,479.34 in total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(session 101). MISSOURI'S NAMED-HOSPITAL DOLLARS ARE $34,646,479.34.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ToRCH Care Smart Growth IFB (DSS26015-02; nearly $40M, awards up to $5M, open to hospitals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">left the DSS bid table between 2026-10-07 and 10-12 with no award, cancellation or amendment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">published: CLOSED, OUTCOME UNKNOWN.</t>
   </si>
   <si>
     <t xml:space="preserve">state</t>
@@ -236,7 +239,7 @@
     <t xml:space="preserve">NON_HOSPITAL</t>
   </si>
   <si>
-    <t xml:space="preserve">HIGH</t>
+    <t xml:space="preserve">MEDIUM</t>
   </si>
   <si>
     <t xml:space="preserve">Recipient name rule: name states an EMS entity. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work.</t>
@@ -254,6 +257,162 @@
     <t xml:space="preserve">data/evidence/MO/2026-07-24_dss_mih_cp_release.html</t>
   </si>
   <si>
+    <t xml:space="preserve">Citizens Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOSPITAL_OR_SYSTEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHTP Strategic Minor Renovations Program award (DSS; named 2026-09-22, priced on the page by 2026-10-13): minor facility improvements, equipment upgrades and infrastructure at a rural hospital. One of 20 awards making up 'approximately $35 million' ($34,646,479.34 summed).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHTP Strategic Minor Renovations Program</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dss.mo.gov/rhtp-strategic-minor-renovations-program</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTICE_OF_AWARD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRATEGIC_MINOR_RENOVATIONS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAMED_HOSPITAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, CITIZENS MEMORIAL HOSPITAL DISTRICT, Bolivar, CCN 260195. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FEDERAL_RECORD_CMS_HOSPITAL_ENROLLMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSS's own 'Awarded Amount' column on the SMRP page ('A full list of awardees and allocation is below'), as served 2026-10-15 (Last-Modified 2026-10-13). Awarded, not a maximum or a request. The 20 rows sum to $34,646,479.34 against the page's 'approximately $35 million'; the page prints no total. Session 54's $0 rows were REWRITTEN from the page, not patched (session 101).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/MO/2026-10-15_dss_smrp_awardees_priced.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golden Valley Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, GOLDEN VALLEY MEMORIAL HOSPITAL DISTRICT, Clinton, CCN 260175. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">John Fitzgibbon Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, JOHN FITZGIBBON MEMORIAL HOSPITAL INC, Marshall, CCN 260142. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lake Regional Health System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, LAKE REGIONAL HEALTH SYSTEM, Osage Beach, CCN 260186. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northeast Regional Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, KIRKSVILLE MISSOURI HOSPITAL COMPANY LLC dba NORTHEAST REGIONAL MEDICAL CENTER, Kirksville, CCN 260022. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poplar Bluff Regional Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, POPLAR BLUFF REGIONAL MEDICAL CENTER LLC, Poplar Bluff, CCN 260119. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scotland County Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, SCOTLAND COUNTY MEMORIAL HOSPITAL dba SCOTLAND COUNTY HOSPITAL, Memphis, CCN 261310. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas County Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, TEXAS COUNTY MEMORIAL HOSPITAL, Houston, CCN 260024. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bothwell Regional Health Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, BOTHWELL REGIONAL HEALTH CENTER, Sedalia, CCN 260009. Classifier said NONPROFIT_CBO/LOW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cameron Regional Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, CAMERON REGIONAL MEDICAL CENTER INC, Cameron, CCN 260057. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carroll County Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, CARROLL COUNTY MEMORIAL HOSPITAL, Carrollton, CCN 261332. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hannibal Regional Healthcare system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, HANNIBAL REGIONAL HEALTHCARE SYSTEM INC dba HANNIBAL REGIONAL HOSPITAL, Hannibal, CCN 260025. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hermann Area District Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, HERMANN AREA HOSPITAL DISTRICT dba HERMANN AREA DISTRICT HOSPITAL, Hermann, CCN 261314. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missouri Delta Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, MISSOURI DELTA MEDICAL CENTER, Sikeston, CCN 260113. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nevada Regional Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, NEVADA CITY HOSPITAL dba NEVADA REGIONAL MEDICAL CENTER, Nevada, CCN 260061. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phelps County Regional Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, PHELPS COUNTY REGIONAL MEDICAL CENTER dba PHELPS HEALTH, Rolla, CCN 260017. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ray County Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, RAY COUNTY MEMORIAL HOSPITAL, Richmond, CCN 261327. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saint Francis Medical Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, SAINT FRANCIS MEDICAL CENTER, Cape Girardeau, CCN 260183 (NOT Mercy St Francis Hospital, Mountain View -- a different body; the string matches Cape Girardeau exactly). Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salem Memorial District Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, SALEM MEMORIAL HOSPITAL, Salem, CCN 261318 (CMS enrols it as 'SALEM MEMORIAL HOSPITAL'; the page's 'District' is its public form). Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Washington County Memorial Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§10.2 DIRECT: DSS names this hospital among the 20 SMRP awardees ('has awarded ... A full list of awardees is below') and the programme 'helps rural hospitals'. Form: CMS Hospital Enrollment, WASHINGTON COUNTY MEMORIAL HOSPITAL, Potosi, CCN 261308. Classifier said HOSPITAL_OR_SYSTEM/MEDIUM.</t>
+  </si>
+  <si>
     <t xml:space="preserve">hub_number</t>
   </si>
   <si>
@@ -284,9 +443,6 @@
     <t xml:space="preserve">Mosaic Medical Center - Maryville</t>
   </si>
   <si>
-    <t xml:space="preserve">HOSPITAL_OR_SYSTEM</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-07-17</t>
   </si>
   <si>
@@ -308,24 +464,15 @@
     <t xml:space="preserve">Harrison County Community Hospital</t>
   </si>
   <si>
-    <t xml:space="preserve">Cameron Regional Medical Center</t>
-  </si>
-  <si>
     <t xml:space="preserve">HCC Network</t>
   </si>
   <si>
     <t xml:space="preserve">Golden Valley Memorial Healthcare</t>
   </si>
   <si>
-    <t xml:space="preserve">Citizens Memorial Hospital</t>
-  </si>
-  <si>
     <t xml:space="preserve">Freeman Health System</t>
   </si>
   <si>
-    <t xml:space="preserve">MEDIUM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mercy Hospital Aurora</t>
   </si>
   <si>
@@ -338,12 +485,6 @@
     <t xml:space="preserve">Ozarks Healthcare</t>
   </si>
   <si>
-    <t xml:space="preserve">Lake Regional Health System</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bothwell Regional Health Center</t>
-  </si>
-  <si>
     <t xml:space="preserve">Randolph County Caring Community Partnership</t>
   </si>
   <si>
@@ -356,9 +497,6 @@
     <t xml:space="preserve">UNIVERSITY_OR_AHC</t>
   </si>
   <si>
-    <t xml:space="preserve">Scotland County Hospital</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hannibal Regional Health Center</t>
   </si>
   <si>
@@ -368,9 +506,6 @@
     <t xml:space="preserve">Mercy Hospital Washington</t>
   </si>
   <si>
-    <t xml:space="preserve">Hermann Area District Hospital</t>
-  </si>
-  <si>
     <t xml:space="preserve">Phelps County Regional Medical Center (dba Phelps Health)</t>
   </si>
   <si>
@@ -386,9 +521,6 @@
     <t xml:space="preserve">Family Counseling Center, Inc. (dba FCC Behavioral Health)</t>
   </si>
   <si>
-    <t xml:space="preserve">Missouri Delta Medical Center</t>
-  </si>
-  <si>
     <t xml:space="preserve">group</t>
   </si>
   <si>
@@ -407,7 +539,7 @@
     <t xml:space="preserve">NOT_AN_AWARD_GOVERNANCE_ROLE</t>
   </si>
   <si>
-    <t xml:space="preserve">RCJ files all 27 ToRCH Care Hub Anchors as Tier 3 award records, each with an amount of $1. They are organisations SELECTED TO CONVENE a hub. DSS's own FAQ: 'Hub Anchors will not act as the fiscal agent' (Q36); its release: participation is 'subject to execution of a Hub Anchor Participation Agreement'. No dollar figure is attached to the role anywhere. 14 of the 27 are hospitals or health systems on the name rule and 11 more carry §8's standing fallback, so believed at face value this publishes at least 14 named hospitals as RHTP recipients with no money behind any.</t>
+    <t xml:space="preserve">RCJ files 27 of the 27 ToRCH Care Hub Anchors as Tier 3 award records, each with an amount of $1. They are organisations SELECTED TO CONVENE a hub. DSS's own FAQ: 'Hub Anchors will not act as the fiscal agent' (Q36); its release: participation is 'subject to execution of a Hub Anchor Participation Agreement'. No dollar figure is attached to the role anywhere. 19 of the 27 are hospitals or health systems on the committed roster (session 49's verification; the name rule alone reaches 14), so believed at face value this publishes 19 named hospitals as RHTP recipients with no money behind any. These rows are unchanged since the 2026-08-27 pull.</t>
   </si>
   <si>
     <t xml:space="preserve">Missouri EMS Association -- a real partnership, amount approximate</t>
@@ -416,16 +548,25 @@
     <t xml:space="preserve">RHTP_AWARD_PASS_THROUGH</t>
   </si>
   <si>
-    <t xml:space="preserve">RCJ's $6,500,000 matches DSS's 'around $6.5M'. It is in this file, as a PASS_THROUGH_UNRESOLVED to rural EMS agencies MEMSA has not named -- not a hospital dollar. WHETHER MEMSA HAS NAMED THEM IS UNKNOWN, NOT NO: https://memsa.org/rht-funding/ answers HTTP 202 with a /.well-known/sgcaptcha/ interstitial, re-tested 2026-09-01 and unchanged. It is NOT a user-agent question -- all four of (project honest (+url), RFC Mozilla/5.0 (compatible), bare Mozilla/5.0, full Chrome) get 202, so §3's michigan.gov exception would not help; robots.txt is itself 202, so no crawler policy is on offer; and the gate needs JavaScript, not a header. Nor is there an archive route: archive.org's availability API answers 200 and returns no snapshot at all, so web.archive.org being unreachable (blocker 7) is not what is in the way -- there is nothing behind it. DO NOT RE-LITIGATE THIS unless testing it deliberately. If it ever answers 200, MEMSA's sub-awardees are a real extraction and still not hospital dollars: DSS states the eligible class and it is rural EMS agencies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missouri Doula Association -- a real award, RCJ's amount short</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RHTP_AWARD_AMOUNT_UNDERSTATED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RCJ carries $732,000 against DSS's own $732,660.43 -- short by $660.43. The award is real and is in this file at the state's figure.</t>
+    <t xml:space="preserve">RCJ's $6,500,000 matches DSS's 'around $6.5M'. It is in this file, as a PASS_THROUGH_UNRESOLVED to rural EMS agencies MEMSA has not named -- not a hospital dollar. RCJ re-keyed it on the 2026-09-24 pull onto an 'Understanding the RHTP' document; one award either way. WHETHER MEMSA HAS NAMED THEM IS UNKNOWN, NOT NO: https://memsa.org/rht-funding/ answers HTTP 202 with a /.well-known/sgcaptcha/ interstitial, re-tested 2026-09-01 and unchanged. It is NOT a user-agent question -- all four of (project honest (+url), RFC Mozilla/5.0 (compatible), bare Mozilla/5.0, full Chrome) get 202, so §3's michigan.gov exception would not help; robots.txt is itself 202, so no crawler policy is on offer; and the gate needs JavaScript, not a header. Nor is there an archive route: archive.org's availability API answers 200 and returns no snapshot at all, so web.archive.org being unreachable (blocker 7) is not what is in the way -- there is nothing behind it. DO NOT RE-LITIGATE THIS unless testing it deliberately. If it ever answers 200, MEMSA's sub-awardees are a real extraction and still not hospital dollars: DSS states the eligible class and it is rural EMS agencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missouri Doula Association -- ONE real award carried on several rows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHTP_AWARD_DUPLICATED_ACROSS_DOCUMENTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCJ carries this one award on 2 rows from 2 documents: 1 at DSS's own $732,660.43 and 1 at $732,000, short by $660.43. Summed, RCJ's rows give $1,464,660.43 for a $732,660.43 award -- §0.1's wrong-grain defect (one row per DOCUMENT, not per award). The award is real and is in this file ONCE, at the state's figure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strategic Minor Renovations Program -- 20 hospital awards RCJ does not carry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT_IN_THE_AGGREGATOR_AT_ALL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSS names 20 rural hospitals as SMRP awardees ('approximately $35 million'), which is CMS's own '20 rural hospital projects' (its 2026-09-22 release); they are in this file as 20 NAMED_HOSPITAL rows (session 54), priced from DSS's 'Awarded Amount' column at $34,646,479.34 (session 101). RCJ carries none of them as a Tier 3 candidate on the 2026-09-24 pull, matched exactly on DSS's spelling. 7 of the 20 SMRP hospitals are also Hub Anchors under the same spelling and appear above only as the $1 anchor rows, which are a different action. A row here means RCJ has caught up and this disposition must be re-read.</t>
   </si>
 </sst>
 </file>
@@ -816,12 +957,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -832,6 +973,11 @@
     <row r="16">
       <c r="A16" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -847,267 +993,1927 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="V1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="X1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Y1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Z1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AA1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AB1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AC1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AD1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D2" t="n">
         <v>732660.43</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="O2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P2"/>
       <c r="Q2"/>
       <c r="R2"/>
       <c r="S2"/>
       <c r="T2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="V2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="W2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Y2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Z2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AA2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AB2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AC2"/>
       <c r="AD2"/>
       <c r="AE2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D3" t="n">
         <v>6500000</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="O3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P3"/>
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3"/>
       <c r="T3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="U3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="V3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="W3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="X3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Y3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Z3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AA3" t="s">
+        <v>75</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" t="s">
+        <v>83</v>
+      </c>
+      <c r="L4" t="s">
+        <v>84</v>
+      </c>
+      <c r="M4" t="s">
+        <v>85</v>
+      </c>
+      <c r="N4" t="s">
+        <v>57</v>
+      </c>
+      <c r="O4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P4"/>
+      <c r="Q4"/>
+      <c r="R4"/>
+      <c r="S4"/>
+      <c r="T4" t="s">
+        <v>86</v>
+      </c>
+      <c r="U4" t="s">
+        <v>87</v>
+      </c>
+      <c r="V4" t="s">
+        <v>88</v>
+      </c>
+      <c r="W4" t="s">
+        <v>52</v>
+      </c>
+      <c r="X4" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y4"/>
+      <c r="Z4" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>78</v>
+      <c r="AA4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC4"/>
+      <c r="AD4" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1272647</v>
+      </c>
+      <c r="E5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" t="s">
+        <v>83</v>
+      </c>
+      <c r="L5" t="s">
+        <v>84</v>
+      </c>
+      <c r="M5" t="s">
+        <v>85</v>
+      </c>
+      <c r="N5" t="s">
+        <v>57</v>
+      </c>
+      <c r="O5" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5"/>
+      <c r="Q5"/>
+      <c r="R5"/>
+      <c r="S5"/>
+      <c r="T5" t="s">
+        <v>86</v>
+      </c>
+      <c r="U5" t="s">
+        <v>87</v>
+      </c>
+      <c r="V5" t="s">
+        <v>88</v>
+      </c>
+      <c r="W5" t="s">
+        <v>52</v>
+      </c>
+      <c r="X5" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y5"/>
+      <c r="Z5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC5"/>
+      <c r="AD5" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2450000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" t="s">
+        <v>53</v>
+      </c>
+      <c r="K6" t="s">
+        <v>83</v>
+      </c>
+      <c r="L6" t="s">
+        <v>84</v>
+      </c>
+      <c r="M6" t="s">
+        <v>85</v>
+      </c>
+      <c r="N6" t="s">
+        <v>57</v>
+      </c>
+      <c r="O6" t="s">
+        <v>58</v>
+      </c>
+      <c r="P6"/>
+      <c r="Q6"/>
+      <c r="R6"/>
+      <c r="S6"/>
+      <c r="T6" t="s">
+        <v>86</v>
+      </c>
+      <c r="U6" t="s">
+        <v>87</v>
+      </c>
+      <c r="V6" t="s">
+        <v>88</v>
+      </c>
+      <c r="W6" t="s">
+        <v>52</v>
+      </c>
+      <c r="X6" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y6"/>
+      <c r="Z6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>97</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC6"/>
+      <c r="AD6" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2482429</v>
+      </c>
+      <c r="E7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H7" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L7" t="s">
+        <v>84</v>
+      </c>
+      <c r="M7" t="s">
+        <v>85</v>
+      </c>
+      <c r="N7" t="s">
+        <v>57</v>
+      </c>
+      <c r="O7" t="s">
+        <v>58</v>
+      </c>
+      <c r="P7"/>
+      <c r="Q7"/>
+      <c r="R7"/>
+      <c r="S7"/>
+      <c r="T7" t="s">
+        <v>86</v>
+      </c>
+      <c r="U7" t="s">
+        <v>87</v>
+      </c>
+      <c r="V7" t="s">
+        <v>88</v>
+      </c>
+      <c r="W7" t="s">
+        <v>52</v>
+      </c>
+      <c r="X7" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y7"/>
+      <c r="Z7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>99</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC7"/>
+      <c r="AD7" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" t="n">
+        <v>216376.59</v>
+      </c>
+      <c r="E8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" t="s">
+        <v>53</v>
+      </c>
+      <c r="K8" t="s">
+        <v>83</v>
+      </c>
+      <c r="L8" t="s">
+        <v>84</v>
+      </c>
+      <c r="M8" t="s">
+        <v>85</v>
+      </c>
+      <c r="N8" t="s">
+        <v>57</v>
+      </c>
+      <c r="O8" t="s">
+        <v>58</v>
+      </c>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8" t="s">
+        <v>86</v>
+      </c>
+      <c r="U8" t="s">
+        <v>87</v>
+      </c>
+      <c r="V8" t="s">
+        <v>88</v>
+      </c>
+      <c r="W8" t="s">
+        <v>52</v>
+      </c>
+      <c r="X8" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y8"/>
+      <c r="Z8" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC8"/>
+      <c r="AD8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" t="n">
+        <v>742416.92</v>
+      </c>
+      <c r="E9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K9" t="s">
+        <v>83</v>
+      </c>
+      <c r="L9" t="s">
+        <v>84</v>
+      </c>
+      <c r="M9" t="s">
+        <v>85</v>
+      </c>
+      <c r="N9" t="s">
+        <v>57</v>
+      </c>
+      <c r="O9" t="s">
+        <v>58</v>
+      </c>
+      <c r="P9"/>
+      <c r="Q9"/>
+      <c r="R9"/>
+      <c r="S9"/>
+      <c r="T9" t="s">
+        <v>86</v>
+      </c>
+      <c r="U9" t="s">
+        <v>87</v>
+      </c>
+      <c r="V9" t="s">
+        <v>88</v>
+      </c>
+      <c r="W9" t="s">
+        <v>52</v>
+      </c>
+      <c r="X9" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y9"/>
+      <c r="Z9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>103</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC9"/>
+      <c r="AD9" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2233540.12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" t="s">
+        <v>53</v>
+      </c>
+      <c r="K10" t="s">
+        <v>83</v>
+      </c>
+      <c r="L10" t="s">
+        <v>84</v>
+      </c>
+      <c r="M10" t="s">
+        <v>85</v>
+      </c>
+      <c r="N10" t="s">
+        <v>57</v>
+      </c>
+      <c r="O10" t="s">
+        <v>58</v>
+      </c>
+      <c r="P10"/>
+      <c r="Q10"/>
+      <c r="R10"/>
+      <c r="S10"/>
+      <c r="T10" t="s">
+        <v>86</v>
+      </c>
+      <c r="U10" t="s">
+        <v>87</v>
+      </c>
+      <c r="V10" t="s">
+        <v>88</v>
+      </c>
+      <c r="W10" t="s">
+        <v>52</v>
+      </c>
+      <c r="X10" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y10"/>
+      <c r="Z10" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC10"/>
+      <c r="AD10" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" t="n">
+        <v>568898.74</v>
+      </c>
+      <c r="E11" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" t="s">
+        <v>82</v>
+      </c>
+      <c r="H11" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" t="s">
+        <v>53</v>
+      </c>
+      <c r="K11" t="s">
+        <v>83</v>
+      </c>
+      <c r="L11" t="s">
+        <v>84</v>
+      </c>
+      <c r="M11" t="s">
+        <v>85</v>
+      </c>
+      <c r="N11" t="s">
+        <v>57</v>
+      </c>
+      <c r="O11" t="s">
+        <v>58</v>
+      </c>
+      <c r="P11"/>
+      <c r="Q11"/>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11" t="s">
+        <v>86</v>
+      </c>
+      <c r="U11" t="s">
+        <v>87</v>
+      </c>
+      <c r="V11" t="s">
+        <v>88</v>
+      </c>
+      <c r="W11" t="s">
+        <v>52</v>
+      </c>
+      <c r="X11" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y11"/>
+      <c r="Z11" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>107</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC11"/>
+      <c r="AD11" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2409200</v>
+      </c>
+      <c r="E12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" t="s">
+        <v>82</v>
+      </c>
+      <c r="H12" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" t="s">
+        <v>52</v>
+      </c>
+      <c r="J12" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" t="s">
+        <v>83</v>
+      </c>
+      <c r="L12" t="s">
+        <v>84</v>
+      </c>
+      <c r="M12" t="s">
+        <v>85</v>
+      </c>
+      <c r="N12" t="s">
+        <v>57</v>
+      </c>
+      <c r="O12" t="s">
+        <v>58</v>
+      </c>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12" t="s">
+        <v>86</v>
+      </c>
+      <c r="U12" t="s">
+        <v>87</v>
+      </c>
+      <c r="V12" t="s">
+        <v>88</v>
+      </c>
+      <c r="W12" t="s">
+        <v>52</v>
+      </c>
+      <c r="X12" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y12"/>
+      <c r="Z12" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC12"/>
+      <c r="AD12" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" t="n">
+        <v>574200</v>
+      </c>
+      <c r="E13" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>82</v>
+      </c>
+      <c r="H13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" t="s">
+        <v>52</v>
+      </c>
+      <c r="J13" t="s">
+        <v>53</v>
+      </c>
+      <c r="K13" t="s">
+        <v>83</v>
+      </c>
+      <c r="L13" t="s">
+        <v>84</v>
+      </c>
+      <c r="M13" t="s">
+        <v>85</v>
+      </c>
+      <c r="N13" t="s">
+        <v>57</v>
+      </c>
+      <c r="O13" t="s">
+        <v>58</v>
+      </c>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13" t="s">
+        <v>86</v>
+      </c>
+      <c r="U13" t="s">
+        <v>87</v>
+      </c>
+      <c r="V13" t="s">
+        <v>88</v>
+      </c>
+      <c r="W13" t="s">
+        <v>52</v>
+      </c>
+      <c r="X13" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y13"/>
+      <c r="Z13" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC13"/>
+      <c r="AD13" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2175000</v>
+      </c>
+      <c r="E14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" t="s">
+        <v>52</v>
+      </c>
+      <c r="J14" t="s">
+        <v>53</v>
+      </c>
+      <c r="K14" t="s">
+        <v>83</v>
+      </c>
+      <c r="L14" t="s">
+        <v>84</v>
+      </c>
+      <c r="M14" t="s">
+        <v>85</v>
+      </c>
+      <c r="N14" t="s">
+        <v>57</v>
+      </c>
+      <c r="O14" t="s">
+        <v>58</v>
+      </c>
+      <c r="P14"/>
+      <c r="Q14"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14" t="s">
+        <v>86</v>
+      </c>
+      <c r="U14" t="s">
+        <v>87</v>
+      </c>
+      <c r="V14" t="s">
+        <v>88</v>
+      </c>
+      <c r="W14" t="s">
+        <v>52</v>
+      </c>
+      <c r="X14" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y14"/>
+      <c r="Z14" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC14"/>
+      <c r="AD14" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15" t="n">
+        <v>439650.76</v>
+      </c>
+      <c r="E15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>82</v>
+      </c>
+      <c r="H15" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" t="s">
+        <v>52</v>
+      </c>
+      <c r="J15" t="s">
+        <v>53</v>
+      </c>
+      <c r="K15" t="s">
+        <v>83</v>
+      </c>
+      <c r="L15" t="s">
+        <v>84</v>
+      </c>
+      <c r="M15" t="s">
+        <v>85</v>
+      </c>
+      <c r="N15" t="s">
+        <v>57</v>
+      </c>
+      <c r="O15" t="s">
+        <v>58</v>
+      </c>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15" t="s">
+        <v>86</v>
+      </c>
+      <c r="U15" t="s">
+        <v>87</v>
+      </c>
+      <c r="V15" t="s">
+        <v>88</v>
+      </c>
+      <c r="W15" t="s">
+        <v>52</v>
+      </c>
+      <c r="X15" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y15"/>
+      <c r="Z15" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC15"/>
+      <c r="AD15" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>116</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1894539</v>
+      </c>
+      <c r="E16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" t="s">
+        <v>82</v>
+      </c>
+      <c r="H16" t="s">
+        <v>52</v>
+      </c>
+      <c r="I16" t="s">
+        <v>52</v>
+      </c>
+      <c r="J16" t="s">
+        <v>53</v>
+      </c>
+      <c r="K16" t="s">
+        <v>83</v>
+      </c>
+      <c r="L16" t="s">
+        <v>84</v>
+      </c>
+      <c r="M16" t="s">
+        <v>85</v>
+      </c>
+      <c r="N16" t="s">
+        <v>57</v>
+      </c>
+      <c r="O16" t="s">
+        <v>58</v>
+      </c>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16" t="s">
+        <v>86</v>
+      </c>
+      <c r="U16" t="s">
+        <v>87</v>
+      </c>
+      <c r="V16" t="s">
+        <v>88</v>
+      </c>
+      <c r="W16" t="s">
+        <v>52</v>
+      </c>
+      <c r="X16" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y16"/>
+      <c r="Z16" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>117</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC16"/>
+      <c r="AD16" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2380000</v>
+      </c>
+      <c r="E17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" t="s">
+        <v>52</v>
+      </c>
+      <c r="I17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J17" t="s">
+        <v>53</v>
+      </c>
+      <c r="K17" t="s">
+        <v>83</v>
+      </c>
+      <c r="L17" t="s">
+        <v>84</v>
+      </c>
+      <c r="M17" t="s">
+        <v>85</v>
+      </c>
+      <c r="N17" t="s">
+        <v>57</v>
+      </c>
+      <c r="O17" t="s">
+        <v>58</v>
+      </c>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17" t="s">
+        <v>86</v>
+      </c>
+      <c r="U17" t="s">
+        <v>87</v>
+      </c>
+      <c r="V17" t="s">
+        <v>88</v>
+      </c>
+      <c r="W17" t="s">
+        <v>52</v>
+      </c>
+      <c r="X17" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y17"/>
+      <c r="Z17" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>119</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC17"/>
+      <c r="AD17" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2431684</v>
+      </c>
+      <c r="E18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" t="s">
+        <v>82</v>
+      </c>
+      <c r="H18" t="s">
+        <v>52</v>
+      </c>
+      <c r="I18" t="s">
+        <v>52</v>
+      </c>
+      <c r="J18" t="s">
+        <v>53</v>
+      </c>
+      <c r="K18" t="s">
+        <v>83</v>
+      </c>
+      <c r="L18" t="s">
+        <v>84</v>
+      </c>
+      <c r="M18" t="s">
+        <v>85</v>
+      </c>
+      <c r="N18" t="s">
+        <v>57</v>
+      </c>
+      <c r="O18" t="s">
+        <v>58</v>
+      </c>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18" t="s">
+        <v>86</v>
+      </c>
+      <c r="U18" t="s">
+        <v>87</v>
+      </c>
+      <c r="V18" t="s">
+        <v>88</v>
+      </c>
+      <c r="W18" t="s">
+        <v>52</v>
+      </c>
+      <c r="X18" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y18"/>
+      <c r="Z18" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC18"/>
+      <c r="AD18" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1529100</v>
+      </c>
+      <c r="E19" t="s">
+        <v>81</v>
+      </c>
+      <c r="F19" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" t="s">
+        <v>52</v>
+      </c>
+      <c r="J19" t="s">
+        <v>53</v>
+      </c>
+      <c r="K19" t="s">
+        <v>83</v>
+      </c>
+      <c r="L19" t="s">
+        <v>84</v>
+      </c>
+      <c r="M19" t="s">
+        <v>85</v>
+      </c>
+      <c r="N19" t="s">
+        <v>57</v>
+      </c>
+      <c r="O19" t="s">
+        <v>58</v>
+      </c>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19" t="s">
+        <v>86</v>
+      </c>
+      <c r="U19" t="s">
+        <v>87</v>
+      </c>
+      <c r="V19" t="s">
+        <v>88</v>
+      </c>
+      <c r="W19" t="s">
+        <v>52</v>
+      </c>
+      <c r="X19" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y19"/>
+      <c r="Z19" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC19"/>
+      <c r="AD19" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1808703.71</v>
+      </c>
+      <c r="E20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" t="s">
+        <v>52</v>
+      </c>
+      <c r="G20" t="s">
+        <v>82</v>
+      </c>
+      <c r="H20" t="s">
+        <v>52</v>
+      </c>
+      <c r="I20" t="s">
+        <v>52</v>
+      </c>
+      <c r="J20" t="s">
+        <v>53</v>
+      </c>
+      <c r="K20" t="s">
+        <v>83</v>
+      </c>
+      <c r="L20" t="s">
+        <v>84</v>
+      </c>
+      <c r="M20" t="s">
+        <v>85</v>
+      </c>
+      <c r="N20" t="s">
+        <v>57</v>
+      </c>
+      <c r="O20" t="s">
+        <v>58</v>
+      </c>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20" t="s">
+        <v>86</v>
+      </c>
+      <c r="U20" t="s">
+        <v>87</v>
+      </c>
+      <c r="V20" t="s">
+        <v>88</v>
+      </c>
+      <c r="W20" t="s">
+        <v>52</v>
+      </c>
+      <c r="X20" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y20"/>
+      <c r="Z20" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>125</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC20"/>
+      <c r="AD20" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>126</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E21" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" t="s">
+        <v>52</v>
+      </c>
+      <c r="G21" t="s">
+        <v>82</v>
+      </c>
+      <c r="H21" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" t="s">
+        <v>52</v>
+      </c>
+      <c r="J21" t="s">
+        <v>53</v>
+      </c>
+      <c r="K21" t="s">
+        <v>83</v>
+      </c>
+      <c r="L21" t="s">
+        <v>84</v>
+      </c>
+      <c r="M21" t="s">
+        <v>85</v>
+      </c>
+      <c r="N21" t="s">
+        <v>57</v>
+      </c>
+      <c r="O21" t="s">
+        <v>58</v>
+      </c>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21" t="s">
+        <v>86</v>
+      </c>
+      <c r="U21" t="s">
+        <v>87</v>
+      </c>
+      <c r="V21" t="s">
+        <v>88</v>
+      </c>
+      <c r="W21" t="s">
+        <v>52</v>
+      </c>
+      <c r="X21" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y21"/>
+      <c r="Z21" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>127</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC21"/>
+      <c r="AD21" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1700599.5</v>
+      </c>
+      <c r="E22" t="s">
+        <v>81</v>
+      </c>
+      <c r="F22" t="s">
+        <v>52</v>
+      </c>
+      <c r="G22" t="s">
+        <v>82</v>
+      </c>
+      <c r="H22" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" t="s">
+        <v>52</v>
+      </c>
+      <c r="J22" t="s">
+        <v>53</v>
+      </c>
+      <c r="K22" t="s">
+        <v>83</v>
+      </c>
+      <c r="L22" t="s">
+        <v>84</v>
+      </c>
+      <c r="M22" t="s">
+        <v>85</v>
+      </c>
+      <c r="N22" t="s">
+        <v>57</v>
+      </c>
+      <c r="O22" t="s">
+        <v>58</v>
+      </c>
+      <c r="P22"/>
+      <c r="Q22"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22" t="s">
+        <v>86</v>
+      </c>
+      <c r="U22" t="s">
+        <v>87</v>
+      </c>
+      <c r="V22" t="s">
+        <v>88</v>
+      </c>
+      <c r="W22" t="s">
+        <v>52</v>
+      </c>
+      <c r="X22" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y22"/>
+      <c r="Z22" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC22"/>
+      <c r="AD22" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
+        <v>130</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2337494</v>
+      </c>
+      <c r="E23" t="s">
+        <v>81</v>
+      </c>
+      <c r="F23" t="s">
+        <v>52</v>
+      </c>
+      <c r="G23" t="s">
+        <v>82</v>
+      </c>
+      <c r="H23" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" t="s">
+        <v>52</v>
+      </c>
+      <c r="J23" t="s">
+        <v>53</v>
+      </c>
+      <c r="K23" t="s">
+        <v>83</v>
+      </c>
+      <c r="L23" t="s">
+        <v>84</v>
+      </c>
+      <c r="M23" t="s">
+        <v>85</v>
+      </c>
+      <c r="N23" t="s">
+        <v>57</v>
+      </c>
+      <c r="O23" t="s">
+        <v>58</v>
+      </c>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23" t="s">
+        <v>86</v>
+      </c>
+      <c r="U23" t="s">
+        <v>87</v>
+      </c>
+      <c r="V23" t="s">
+        <v>88</v>
+      </c>
+      <c r="W23" t="s">
+        <v>52</v>
+      </c>
+      <c r="X23" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y23"/>
+      <c r="Z23" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>131</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC23"/>
+      <c r="AD23" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1123,618 +2929,618 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="C1" t="s">
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="D1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" t="s">
-        <v>81</v>
+        <v>134</v>
       </c>
       <c r="F1" t="s">
-        <v>82</v>
+        <v>135</v>
       </c>
       <c r="G1" t="s">
-        <v>83</v>
+        <v>136</v>
       </c>
       <c r="H1" t="s">
-        <v>84</v>
+        <v>137</v>
       </c>
       <c r="I1" t="s">
-        <v>85</v>
+        <v>138</v>
       </c>
       <c r="J1" t="s">
-        <v>86</v>
+        <v>139</v>
       </c>
       <c r="K1" t="s">
-        <v>87</v>
+        <v>140</v>
       </c>
       <c r="L1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>141</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K2" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L2" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M2" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O2" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>147</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K3" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L3" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M3" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O3" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K4" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L4" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M4" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O4" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K5" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L5" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M5" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O5" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>149</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K6" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L6" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M6" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O6" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F7" t="b">
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K7" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L7" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M7" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O7" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K8" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L8" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M8" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O8" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>151</v>
       </c>
       <c r="D9" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E9" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K9" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L9" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M9" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O9" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>152</v>
       </c>
       <c r="D10" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K10" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L10" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M10" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O10" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>153</v>
       </c>
       <c r="D11" t="s">
-        <v>105</v>
+        <v>154</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K11" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L11" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M11" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O11" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F12" t="b">
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K12" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L12" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M12" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O12" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K13" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L13" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M13" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O13" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B14" t="n">
         <v>13</v>
@@ -1743,698 +3549,698 @@
         <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K14" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L14" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M14" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O14" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>156</v>
       </c>
       <c r="D15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
       </c>
       <c r="G15" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K15" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L15" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M15" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O15" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>157</v>
       </c>
       <c r="D16" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K16" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L16" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M16" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O16" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>158</v>
       </c>
       <c r="D17" t="s">
-        <v>112</v>
+        <v>159</v>
       </c>
       <c r="E17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K17" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L17" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M17" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O17" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
       </c>
       <c r="G18" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K18" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L18" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M18" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O18" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>160</v>
       </c>
       <c r="D19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K19" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L19" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M19" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O19" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="s">
-        <v>115</v>
+        <v>161</v>
       </c>
       <c r="D20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
       </c>
       <c r="G20" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K20" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L20" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M20" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O20" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>116</v>
+        <v>162</v>
       </c>
       <c r="D21" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K21" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L21" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M21" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O21" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K22" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L22" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M22" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O22" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>163</v>
       </c>
       <c r="D23" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K23" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L23" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M23" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O23" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>119</v>
+        <v>164</v>
       </c>
       <c r="D24" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E24" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K24" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L24" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M24" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O24" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="D25" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E25" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
       </c>
       <c r="G25" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K25" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L25" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M25" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N25" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O25" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>166</v>
       </c>
       <c r="D26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
       </c>
       <c r="G26" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K26" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L26" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M26" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O26" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>122</v>
+        <v>167</v>
       </c>
       <c r="D27" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E27" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
       </c>
       <c r="G27" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K27" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L27" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M27" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N27" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O27" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D28" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F28" t="b">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K28" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="L28" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="M28" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="N28" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O28" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2450,70 +4256,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>168</v>
       </c>
       <c r="C1" t="s">
-        <v>125</v>
+        <v>169</v>
       </c>
       <c r="D1" t="s">
-        <v>126</v>
+        <v>170</v>
       </c>
       <c r="E1" t="s">
-        <v>127</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>172</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>129</v>
+        <v>173</v>
       </c>
       <c r="E2" t="s">
-        <v>130</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>175</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>132</v>
+        <v>176</v>
       </c>
       <c r="E3" t="s">
-        <v>133</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
+        <v>178</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>135</v>
+        <v>179</v>
       </c>
       <c r="E4" t="s">
-        <v>136</v>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>